<commit_message>
Sync data files - 2025-08-07 10:45:18 (       4 files updated)
</commit_message>
<xml_diff>
--- a/Data/Listings/sidra.xlsx
+++ b/Data/Listings/sidra.xlsx
@@ -19,13 +19,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <color rgb="00FF0000"/>
     </font>
     <font>
       <color rgb="00008000"/>
@@ -72,16 +75,17 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -448,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U113"/>
+  <dimension ref="A1:U114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -654,7 +658,7 @@
         </is>
       </c>
       <c r="Q2" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -764,7 +768,7 @@
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -879,7 +883,7 @@
         </is>
       </c>
       <c r="Q4" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -999,7 +1003,7 @@
         </is>
       </c>
       <c r="Q5" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -1109,7 +1113,7 @@
         </is>
       </c>
       <c r="Q6" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1229,7 +1233,7 @@
         </is>
       </c>
       <c r="Q7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -1338,7 +1342,7 @@
         </is>
       </c>
       <c r="Q8" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1446,7 +1450,7 @@
         </is>
       </c>
       <c r="Q9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -1542,7 +1546,7 @@
         </is>
       </c>
       <c r="Q10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -1653,7 +1657,7 @@
         </is>
       </c>
       <c r="Q11" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -1770,7 +1774,7 @@
         </is>
       </c>
       <c r="Q12" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -1877,7 +1881,7 @@
         </is>
       </c>
       <c r="Q13" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
@@ -1985,7 +1989,7 @@
         </is>
       </c>
       <c r="Q14" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
@@ -2093,7 +2097,7 @@
         </is>
       </c>
       <c r="Q15" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
@@ -2200,7 +2204,7 @@
         </is>
       </c>
       <c r="Q16" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
@@ -2304,7 +2308,7 @@
         </is>
       </c>
       <c r="Q17" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
@@ -2406,7 +2410,7 @@
         </is>
       </c>
       <c r="Q18" t="n">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
@@ -2502,7 +2506,7 @@
         </is>
       </c>
       <c r="Q19" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
@@ -2521,7 +2525,8 @@
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>Brought to you by Driven Properties, this 5 Bedroom Villa is located in Sidra Villas II, Dubai Hills Estate.
+          <t xml:space="preserve">
+Brought to you by Driven Properties, this 5 Bedroom Villa is located in Sidra Villas II, Dubai Hills Estate.
 Unit Details:
   * Vacant Villa 
   * Unit Type: E5 
@@ -2556,7 +2561,8 @@
   * Business Bay
   * Dubai Creek Harbour
   * Jumeirah Village Circle
-  * Dubai Hills Estate</t>
+  * Dubai Hills Estate
+</t>
         </is>
       </c>
     </row>
@@ -2628,7 +2634,7 @@
         </is>
       </c>
       <c r="Q20" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
@@ -2742,7 +2748,7 @@
         </is>
       </c>
       <c r="Q21" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
@@ -2849,7 +2855,7 @@
         </is>
       </c>
       <c r="Q22" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
@@ -2958,7 +2964,7 @@
         </is>
       </c>
       <c r="Q23" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
@@ -3073,7 +3079,7 @@
         </is>
       </c>
       <c r="Q24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
@@ -3197,7 +3203,7 @@
         </is>
       </c>
       <c r="Q25" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
@@ -3306,7 +3312,7 @@
         </is>
       </c>
       <c r="Q26" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="R26" t="inlineStr">
         <is>
@@ -3417,7 +3423,7 @@
         </is>
       </c>
       <c r="Q27" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="R27" t="inlineStr">
         <is>
@@ -3525,7 +3531,7 @@
         </is>
       </c>
       <c r="Q28" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
@@ -3634,7 +3640,7 @@
         </is>
       </c>
       <c r="Q29" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
@@ -3744,7 +3750,7 @@
         </is>
       </c>
       <c r="Q30" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
@@ -3852,7 +3858,7 @@
         </is>
       </c>
       <c r="Q31" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="R31" t="inlineStr">
         <is>
@@ -3963,7 +3969,7 @@
         </is>
       </c>
       <c r="Q32" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R32" t="inlineStr">
         <is>
@@ -4072,7 +4078,7 @@
         </is>
       </c>
       <c r="Q33" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="R33" t="inlineStr">
         <is>
@@ -4182,7 +4188,7 @@
         </is>
       </c>
       <c r="Q34" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R34" t="inlineStr">
         <is>
@@ -4284,7 +4290,7 @@
         </is>
       </c>
       <c r="Q35" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="R35" t="inlineStr">
         <is>
@@ -4405,7 +4411,7 @@
         </is>
       </c>
       <c r="Q36" t="n">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="R36" t="inlineStr">
         <is>
@@ -4501,7 +4507,7 @@
         </is>
       </c>
       <c r="Q37" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="R37" t="inlineStr">
         <is>
@@ -4597,7 +4603,7 @@
         </is>
       </c>
       <c r="Q38" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="R38" t="inlineStr">
         <is>
@@ -4693,7 +4699,7 @@
         </is>
       </c>
       <c r="Q39" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R39" t="inlineStr">
         <is>
@@ -4792,7 +4798,7 @@
         </is>
       </c>
       <c r="Q40" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="R40" t="inlineStr">
         <is>
@@ -4902,7 +4908,7 @@
         </is>
       </c>
       <c r="Q41" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="R41" t="inlineStr">
         <is>
@@ -5020,7 +5026,7 @@
         </is>
       </c>
       <c r="Q42" t="n">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="R42" t="inlineStr">
         <is>
@@ -5131,7 +5137,7 @@
         </is>
       </c>
       <c r="Q43" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="R43" t="inlineStr">
         <is>
@@ -5238,7 +5244,7 @@
         </is>
       </c>
       <c r="Q44" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R44" t="inlineStr">
         <is>
@@ -5350,7 +5356,7 @@
         </is>
       </c>
       <c r="Q45" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R45" t="inlineStr">
         <is>
@@ -5461,7 +5467,7 @@
         </is>
       </c>
       <c r="Q46" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="R46" t="inlineStr">
         <is>
@@ -5558,7 +5564,7 @@
         </is>
       </c>
       <c r="Q47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R47" t="inlineStr">
         <is>
@@ -5660,7 +5666,7 @@
         </is>
       </c>
       <c r="Q48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R48" t="inlineStr">
         <is>
@@ -5765,7 +5771,7 @@
         </is>
       </c>
       <c r="Q49" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="R49" t="inlineStr">
         <is>
@@ -5873,7 +5879,7 @@
         </is>
       </c>
       <c r="Q50" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R50" t="inlineStr">
         <is>
@@ -5913,7 +5919,7 @@
           <t>L-800</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>6531921899</t>
         </is>
@@ -5975,7 +5981,7 @@
         </is>
       </c>
       <c r="Q51" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="R51" t="inlineStr">
         <is>
@@ -6085,7 +6091,7 @@
         </is>
       </c>
       <c r="Q52" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="R52" t="inlineStr">
         <is>
@@ -6128,94 +6134,201 @@
     <row r="53">
       <c r="A53" s="1" t="inlineStr">
         <is>
+          <t>L-9009</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>6529103221</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.propertyfinder.ae/en/plp/buy/villa-for-sale-dubai-dubai-hills-estate-sidra-villas-sidra-villas-i-14890412.html</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Dubai Hills Estate</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Sidra Villas</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Sidra Villas I</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>10500000</v>
+      </c>
+      <c r="I53" t="n">
+        <v>3</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Villa</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Type E1</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>3100</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>Exclusive Luxury Villa | Private Pool | E1</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>2025-08-05</t>
+        </is>
+      </c>
+      <c r="Q53" t="n">
+        <v>2</v>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Peter Delargey</t>
+        </is>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>EQUITY REAL ESTATES L.L.C</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>Equity wants you to experience a luxurious living space meticulously upgraded to offer an unparalleled lifestyle in Sidra Villa, Dubai Hills Estate.
+- 3 Bedroom + Maids
+- Fully Upgraded
+- Stunning Finishing
+- Highest Quality Upgrades
+- Single Road
+- Vacant On Transfer
+- Plot 4,486.61 Sq Ft
+- Open Plan Living, Kitchen and Dining
+- Permit No.: 6529103221
+The interior offers an extended living, kitchen, and dining area designed for both comfort and elegance, featuring a flush ceiling with modern lighting and pristine high-end furniture. A striking TV wall unit with a 3D fireplace adds warmth and sophistication, making it perfect for cozy gatherings.
+Step outside to a private outdoor sanctuary with a luxurious overflow pool, refreshing shower, and a stylish dining area complete with an electric awning for shade. A sleek aluminum pergola and marble-finished bar complete the space, ideal for relaxing or entertaining in style.
+Please be advised that all measurements and information are provided to the best of our knowledge. Equity disclaims any liability for inaccuracies or discrepancies.
+Equity
+RERA ORN: 43321
+Address: Office 1902, Boulevard Plaza Tower 2, Downtown Dubai, Dubai, UAE</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
           <t>LIV-S-1267</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>6544322776</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>https://www.propertyfinder.ae/en/plp/buy/villa-for-sale-dubai-dubai-hills-estate-sidra-villas-sidra-villas-ii-14600503.html</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>Dubai Hills Estate</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>Sidra Villas</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>Sidra Villas II</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G54" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H53" t="n">
+      <c r="H54" t="n">
         <v>15350000</v>
       </c>
-      <c r="I53" t="n">
+      <c r="I54" t="n">
         <v>4</v>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="J54" t="inlineStr">
         <is>
           <t>Villa</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr">
+      <c r="K54" t="inlineStr">
         <is>
           <t>Type E3</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr">
+      <c r="M54" t="inlineStr">
         <is>
           <t>3533</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr">
+      <c r="N54" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="O53" t="inlineStr">
+      <c r="O54" t="inlineStr">
         <is>
           <t>Premium Upgraded / Extended / Private Pool</t>
         </is>
       </c>
-      <c r="P53" t="inlineStr">
+      <c r="P54" t="inlineStr">
         <is>
           <t>2025-06-26</t>
         </is>
       </c>
-      <c r="Q53" t="n">
-        <v>41</v>
-      </c>
-      <c r="R53" t="inlineStr">
+      <c r="Q54" t="n">
+        <v>42</v>
+      </c>
+      <c r="R54" t="inlineStr">
         <is>
           <t>Iana Varyvoda</t>
         </is>
       </c>
-      <c r="S53" t="inlineStr">
+      <c r="S54" t="inlineStr">
         <is>
           <t>Livrichy Real Estate Brokerage - Business Bay</t>
         </is>
       </c>
-      <c r="T53" t="inlineStr">
+      <c r="T54" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
       </c>
-      <c r="U53" t="inlineStr">
+      <c r="U54" t="inlineStr">
         <is>
           <t xml:space="preserve">Livrichy Real Estate is delighted to present this elegant villa for sale located in the highly sought-after Sidra 2 community within Dubai Hills Estate.
 Property Details:
@@ -6241,116 +6354,20 @@
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="1" t="inlineStr">
-        <is>
-          <t>LP45347</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>65102648580</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>https://www.propertyfinder.ae/en/plp/buy/villa-for-sale-dubai-dubai-hills-estate-sidra-villas-sidra-villas-iii-14424924.html</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Dubai Hills Estate</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Sidra Villas</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>Sidra Villas III</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H54" t="n">
-        <v>13000000</v>
-      </c>
-      <c r="I54" t="n">
-        <v>4</v>
-      </c>
-      <c r="J54" t="inlineStr">
-        <is>
-          <t>Villa</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>Type E3</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>3533</t>
-        </is>
-      </c>
-      <c r="N54" t="inlineStr">
-        <is>
-          <t>4669</t>
-        </is>
-      </c>
-      <c r="O54" t="inlineStr">
-        <is>
-          <t>Exclusive | Elevated Plot | Backing Park</t>
-        </is>
-      </c>
-      <c r="P54" t="inlineStr">
-        <is>
-          <t>2025-06-03</t>
-        </is>
-      </c>
-      <c r="Q54" t="n">
-        <v>64</v>
-      </c>
-      <c r="R54" t="inlineStr">
-        <is>
-          <t>Elijah Crabtree</t>
-        </is>
-      </c>
-      <c r="S54" t="inlineStr">
-        <is>
-          <t>LuxuryProperty.com</t>
-        </is>
-      </c>
-      <c r="T54" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="U54" t="inlineStr">
-        <is>
-          <t>&lt;p&gt;Presented by LuxuryProperty.com, this exclusive four-bedroom villa in Sidra 3, Dubai Hills Estate, sits on an elevated corner plot backing directly onto the park and tennis courts. Boasting open views and a peaceful setting, the villa offers a unique opportunity for families seeking a private, park-facing home in one of Dubais most prestigious communities. &lt;/p&gt;&lt;p&gt; &lt;/p&gt;&lt;p&gt;Key Features:&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;br&gt; 4 Bedrooms, 4 Bathrooms&lt;br&gt; BUA: 3,500 sq. ft.&lt;br&gt; Plot: 4,669 sq. ft.&lt;br&gt; Elevated Corner Plot&lt;br&gt; Direct Park &amp;amp; Tennis Court Views&lt;br&gt; Contemporary Interior Finish&lt;br&gt; Vacant in 4 Weeks&lt;br&gt; Family-Friendly Layout&lt;/li&gt;&lt;/ul&gt;&lt;p&gt; &lt;/p&gt;&lt;p&gt;Sidra 3 is a sought-after sub-community within Dubai Hills Estate, known for its well-planned streets, green landscapes, and easy access to top schools, Dubai Hills Mall, and major roads. Residents enjoy world-class amenities including parks, fitness trails, and golf facilities, making this home an excellent investment for modern family living.&lt;/p&gt;</t>
-        </is>
-      </c>
-    </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr">
         <is>
-          <t>MCC-S-46811</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="inlineStr">
-        <is>
-          <t>6531968111</t>
+          <t>LP45347</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>65102648580</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>https://www.propertyfinder.ae/en/plp/buy/villa-for-sale-dubai-dubai-hills-estate-sidra-villas-sidra-villas-i-14791643.html</t>
+          <t>https://www.propertyfinder.ae/en/plp/buy/villa-for-sale-dubai-dubai-hills-estate-sidra-villas-sidra-villas-iii-14424924.html</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6365,7 +6382,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Sidra Villas I</t>
+          <t>Sidra Villas III</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -6374,7 +6391,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>16500000</v>
+        <v>13000000</v>
       </c>
       <c r="I55" t="n">
         <v>4</v>
@@ -6384,45 +6401,141 @@
           <t>Villa</t>
         </is>
       </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Type E3</t>
+        </is>
+      </c>
       <c r="M55" t="inlineStr">
         <is>
+          <t>3533</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>4669</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>Exclusive | Elevated Plot | Backing Park</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>2025-06-03</t>
+        </is>
+      </c>
+      <c r="Q55" t="n">
+        <v>65</v>
+      </c>
+      <c r="R55" t="inlineStr">
+        <is>
+          <t>Elijah Crabtree</t>
+        </is>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>LuxuryProperty.com</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Presented by LuxuryProperty.com, this exclusive four-bedroom villa in Sidra 3, Dubai Hills Estate, sits on an elevated corner plot backing directly onto the park and tennis courts. Boasting open views and a peaceful setting, the villa offers a unique opportunity for families seeking a private, park-facing home in one of Dubais most prestigious communities. &lt;/p&gt;&lt;p&gt; &lt;/p&gt;&lt;p&gt;Key Features:&lt;/p&gt;&lt;ul&gt;&lt;li&gt;&lt;br&gt; 4 Bedrooms, 4 Bathrooms&lt;br&gt; BUA: 3,500 sq. ft.&lt;br&gt; Plot: 4,669 sq. ft.&lt;br&gt; Elevated Corner Plot&lt;br&gt; Direct Park &amp;amp; Tennis Court Views&lt;br&gt; Contemporary Interior Finish&lt;br&gt; Vacant in 4 Weeks&lt;br&gt; Family-Friendly Layout&lt;/li&gt;&lt;/ul&gt;&lt;p&gt; &lt;/p&gt;&lt;p&gt;Sidra 3 is a sought-after sub-community within Dubai Hills Estate, known for its well-planned streets, green landscapes, and easy access to top schools, Dubai Hills Mall, and major roads. Residents enjoy world-class amenities including parks, fitness trails, and golf facilities, making this home an excellent investment for modern family living.&lt;/p&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>MCC-S-46811</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>6531968111</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>https://www.propertyfinder.ae/en/plp/buy/villa-for-sale-dubai-dubai-hills-estate-sidra-villas-sidra-villas-i-14791643.html</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Dubai Hills Estate</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Sidra Villas</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Sidra Villas I</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>16500000</v>
+      </c>
+      <c r="I56" t="n">
+        <v>4</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>Villa</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
           <t>4650</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr">
+      <c r="N56" t="inlineStr">
         <is>
           <t>4650</t>
         </is>
       </c>
-      <c r="O55" t="inlineStr">
+      <c r="O56" t="inlineStr">
         <is>
           <t>Premium Upgrade | Extended + Maids | Private Pool</t>
         </is>
       </c>
-      <c r="P55" t="inlineStr">
+      <c r="P56" t="inlineStr">
         <is>
           <t>2025-07-21</t>
         </is>
       </c>
-      <c r="Q55" t="n">
-        <v>16</v>
-      </c>
-      <c r="R55" t="inlineStr">
+      <c r="Q56" t="n">
+        <v>17</v>
+      </c>
+      <c r="R56" t="inlineStr">
         <is>
           <t>Faisal Farooqui</t>
         </is>
       </c>
-      <c r="S55" t="inlineStr">
+      <c r="S56" t="inlineStr">
         <is>
           <t>McCone Properties</t>
         </is>
       </c>
-      <c r="T55" t="inlineStr">
+      <c r="T56" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
       </c>
-      <c r="U55" t="inlineStr">
+      <c r="U56" t="inlineStr">
         <is>
           <t>Property Highlights:
 - 4 Bedrooms + Maid’s Room
@@ -6446,114 +6559,6 @@
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="1" t="inlineStr">
-        <is>
-          <t>MDXBSIIIDHE</t>
-        </is>
-      </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t>65102643812</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>https://www.propertyfinder.ae/en/plp/buy/villa-for-sale-dubai-dubai-hills-estate-sidra-villas-sidra-villas-iii-14708936.html</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Dubai Hills Estate</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Sidra Villas</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>Sidra Villas III</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H56" t="n">
-        <v>11200000</v>
-      </c>
-      <c r="I56" t="n">
-        <v>4</v>
-      </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>Villa</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>Type E3</t>
-        </is>
-      </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>3533</t>
-        </is>
-      </c>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>4901</t>
-        </is>
-      </c>
-      <c r="O56" t="inlineStr">
-        <is>
-          <t>Type E3 | Immaculate Condition | Single Row</t>
-        </is>
-      </c>
-      <c r="P56" t="inlineStr">
-        <is>
-          <t>2025-07-09</t>
-        </is>
-      </c>
-      <c r="Q56" t="n">
-        <v>28</v>
-      </c>
-      <c r="R56" t="inlineStr">
-        <is>
-          <t>Conor Davis</t>
-        </is>
-      </c>
-      <c r="S56" t="inlineStr">
-        <is>
-          <t>MONDAY REAL ESTATE L.L.C</t>
-        </is>
-      </c>
-      <c r="T56" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="U56" t="inlineStr">
-        <is>
-          <t>Monday Real Estate is proud to present this beautifully maintained Type E3 villa in the sought-after Sidra Villas III, Dubai Hills Estate. Set on an expansive 4,901 sq. ft. plot, this 4-bedroom villa offers 3,953 sq. ft. of spacious, modern living in immaculate condition.
-The home features a bright and airy open-plan layout, high-quality finishes, and generously sized bedrooms - each with built-in wardrobes and en-suite bathrooms. The landscaped garden provides an ideal space for outdoor living and entertaining.
-Located within one of Dubai’s most prestigious master communities, residents benefit from lush parks, walking trails, top-tier schools, and proximity to Dubai Hills Mall and the golf course.
-Key Features:
-- 4 Bedrooms
-- Maid’s Room
-- 5 Bathrooms
-- Type E3 Layout
-- Immaculately Maintained
-- Large Plot: 4,901 sq. ft.
-- Built-Up Area: 3,953 sq. ft.
-- Family-Friendly Community
-This villa is perfect for families seeking a high-quality lifestyle in a well-connected and vibrant neighbourhood.</t>
-        </is>
-      </c>
-    </row>
     <row r="57">
       <c r="A57" s="1" t="inlineStr">
         <is>
@@ -6627,7 +6632,7 @@
         </is>
       </c>
       <c r="Q57" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="R57" t="inlineStr">
         <is>
@@ -6737,7 +6742,7 @@
         </is>
       </c>
       <c r="Q58" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="R58" t="inlineStr">
         <is>
@@ -6843,7 +6848,7 @@
         </is>
       </c>
       <c r="Q59" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="R59" t="inlineStr">
         <is>
@@ -6956,7 +6961,7 @@
         </is>
       </c>
       <c r="Q60" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R60" t="inlineStr">
         <is>
@@ -7054,7 +7059,7 @@
         </is>
       </c>
       <c r="Q61" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R61" t="inlineStr">
         <is>
@@ -7161,7 +7166,7 @@
         </is>
       </c>
       <c r="Q62" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R62" t="inlineStr">
         <is>
@@ -7270,7 +7275,7 @@
         </is>
       </c>
       <c r="Q63" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="R63" t="inlineStr">
         <is>
@@ -7382,7 +7387,7 @@
         </is>
       </c>
       <c r="Q64" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="R64" t="inlineStr">
         <is>
@@ -7495,7 +7500,7 @@
         </is>
       </c>
       <c r="Q65" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R65" t="inlineStr">
         <is>
@@ -7610,7 +7615,7 @@
         </is>
       </c>
       <c r="Q66" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R66" t="inlineStr">
         <is>
@@ -7712,7 +7717,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>Vacant now | Extended | Big Plot | Corner</t>
+          <t>Extended | Corner | Vacant | Single row</t>
         </is>
       </c>
       <c r="P67" t="inlineStr">
@@ -7721,7 +7726,7 @@
         </is>
       </c>
       <c r="Q67" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="R67" t="inlineStr">
         <is>
@@ -7822,7 +7827,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>Owner occupied | On top of the hill | Extended</t>
+          <t>VOT | Fully extended | Spanish tiles</t>
         </is>
       </c>
       <c r="P68" t="inlineStr">
@@ -7831,7 +7836,7 @@
         </is>
       </c>
       <c r="Q68" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R68" t="inlineStr">
         <is>
@@ -7930,7 +7935,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>Big Plot| Type E5| Vacant| Near Pool</t>
+          <t>Vacant| Near Pool| Big Plot| Type E5</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
@@ -7939,7 +7944,7 @@
         </is>
       </c>
       <c r="Q69" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="R69" t="inlineStr">
         <is>
@@ -8056,7 +8061,7 @@
         </is>
       </c>
       <c r="Q70" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="R70" t="inlineStr">
         <is>
@@ -8166,7 +8171,7 @@
         </is>
       </c>
       <c r="Q71" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="R71" t="inlineStr">
         <is>
@@ -8275,7 +8280,7 @@
         </is>
       </c>
       <c r="Q72" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="R72" t="inlineStr">
         <is>
@@ -8388,7 +8393,7 @@
         </is>
       </c>
       <c r="Q73" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R73" t="inlineStr">
         <is>
@@ -8508,7 +8513,7 @@
         </is>
       </c>
       <c r="Q74" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="R74" t="inlineStr">
         <is>
@@ -8619,7 +8624,7 @@
         </is>
       </c>
       <c r="Q75" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="R75" t="inlineStr">
         <is>
@@ -8731,7 +8736,7 @@
         </is>
       </c>
       <c r="Q76" t="n">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="R76" t="inlineStr">
         <is>
@@ -8847,7 +8852,7 @@
         </is>
       </c>
       <c r="Q77" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R77" t="inlineStr">
         <is>
@@ -8968,7 +8973,7 @@
         </is>
       </c>
       <c r="Q78" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="R78" t="inlineStr">
         <is>
@@ -9081,7 +9086,7 @@
         </is>
       </c>
       <c r="Q79" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="R79" t="inlineStr">
         <is>
@@ -9188,7 +9193,7 @@
         </is>
       </c>
       <c r="Q80" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="R80" t="inlineStr">
         <is>
@@ -9291,7 +9296,7 @@
         </is>
       </c>
       <c r="Q81" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="R81" t="inlineStr">
         <is>
@@ -9413,11 +9418,11 @@
         </is>
       </c>
       <c r="Q82" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>Cosmin Laurentiu Dancea (Tomas)</t>
+          <t>Nicole Saletnik</t>
         </is>
       </c>
       <c r="S82" t="inlineStr">
@@ -9526,7 +9531,7 @@
         </is>
       </c>
       <c r="Q83" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R83" t="inlineStr">
         <is>
@@ -9641,7 +9646,7 @@
         </is>
       </c>
       <c r="Q84" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R84" t="inlineStr">
         <is>
@@ -9751,7 +9756,7 @@
         </is>
       </c>
       <c r="Q85" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="R85" t="inlineStr">
         <is>
@@ -9868,7 +9873,7 @@
         </is>
       </c>
       <c r="Q86" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="R86" t="inlineStr">
         <is>
@@ -9972,7 +9977,7 @@
         </is>
       </c>
       <c r="Q87" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="R87" t="inlineStr">
         <is>
@@ -10085,7 +10090,7 @@
         </is>
       </c>
       <c r="Q88" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="R88" t="inlineStr">
         <is>
@@ -10184,7 +10189,7 @@
         </is>
       </c>
       <c r="Q89" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="R89" t="inlineStr">
         <is>
@@ -10292,7 +10297,7 @@
         </is>
       </c>
       <c r="Q90" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R90" t="inlineStr">
         <is>
@@ -10401,7 +10406,7 @@
         </is>
       </c>
       <c r="Q91" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R91" t="inlineStr">
         <is>
@@ -10509,7 +10514,7 @@
         </is>
       </c>
       <c r="Q92" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="R92" t="inlineStr">
         <is>
@@ -10615,7 +10620,7 @@
         </is>
       </c>
       <c r="Q93" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="R93" t="inlineStr">
         <is>
@@ -10724,7 +10729,7 @@
         </is>
       </c>
       <c r="Q94" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="R94" t="inlineStr">
         <is>
@@ -10832,7 +10837,7 @@
         </is>
       </c>
       <c r="Q95" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="R95" t="inlineStr">
         <is>
@@ -10934,7 +10939,7 @@
         </is>
       </c>
       <c r="Q96" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R96" t="inlineStr">
         <is>
@@ -11039,7 +11044,7 @@
         </is>
       </c>
       <c r="Q97" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R97" t="inlineStr">
         <is>
@@ -11149,7 +11154,7 @@
         </is>
       </c>
       <c r="Q98" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="R98" t="inlineStr">
         <is>
@@ -11259,7 +11264,7 @@
         </is>
       </c>
       <c r="Q99" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="R99" t="inlineStr">
         <is>
@@ -11364,7 +11369,7 @@
         </is>
       </c>
       <c r="Q100" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R100" t="inlineStr">
         <is>
@@ -11478,7 +11483,7 @@
         </is>
       </c>
       <c r="Q101" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="R101" t="inlineStr">
         <is>
@@ -11595,7 +11600,7 @@
         </is>
       </c>
       <c r="Q102" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="R102" t="inlineStr">
         <is>
@@ -11697,7 +11702,7 @@
         </is>
       </c>
       <c r="Q103" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R103" t="inlineStr">
         <is>
@@ -11805,7 +11810,7 @@
         </is>
       </c>
       <c r="Q104" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="R104" t="inlineStr">
         <is>
@@ -11913,7 +11918,7 @@
         </is>
       </c>
       <c r="Q105" t="n">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="R105" t="inlineStr">
         <is>
@@ -12016,7 +12021,7 @@
         </is>
       </c>
       <c r="Q106" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="R106" t="inlineStr">
         <is>
@@ -12136,11 +12141,11 @@
         </is>
       </c>
       <c r="Q107" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="R107" t="inlineStr">
         <is>
-          <t>Keisha Convento</t>
+          <t>Waqas Abbassi Zafar Mehmood</t>
         </is>
       </c>
       <c r="S107" t="inlineStr">
@@ -12173,94 +12178,199 @@
     <row r="108">
       <c r="A108" s="1" t="inlineStr">
         <is>
+          <t>luxure-14092927</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>65102648813</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>https://www.propertyfinder.ae/en/plp/buy/villa-for-sale-dubai-dubai-hills-estate-sidra-villas-sidra-villas-iii-14833599.html</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Dubai Hills Estate</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Sidra Villas</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Sidra Villas III</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H108" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="I108" t="n">
+        <v>5</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Villa</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Type E5</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>4109</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr"/>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>Fullly Upgraded | Furnished | Private Pool</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>2025-07-28</t>
+        </is>
+      </c>
+      <c r="Q108" t="n">
+        <v>10</v>
+      </c>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t>Hibildas Haridas</t>
+        </is>
+      </c>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>THE LUXURY REAL ESTATE BROKER L.L.C</t>
+        </is>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>The Luxury Real Estate is thrilled to present this fully upgraded, spacious, and elegantly furnished 4-bedroom villa with a serene community view in Sidra III, developed by Emaar Properties.
+Property Features:
+- Five Bedrooms
+- Six Bathrooms
+- Size: 4,902.96 SqFt.
+- Balcony with Community View
+- 2 Covered Parking Spaces
+- Fully Upgraded
+- Fully Furnished
+- Private Pool
+- Bright &amp;amp; Spacious
+- Standard Layout
+Located in the prestigious Dubai Hills Estate, this villa offers a tranquil living experience, surrounded by nature&amp;#39;s beauty. The design of Sidra villas incorporates a minimalist architectural style, maximizing natural light and airflow, creating a harmonious and eco-friendly living environment. 
+The Luxury Real Estate (TLRE) is a premier global real estate company specializing in high-end properties. With access to an exclusively owned portfolio, TLRE offers unique, luxury residences to discerning buyers. known for its personalized service and extensive market expertise, it connects clients to exceptional homes worldwide.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="1" t="inlineStr">
+        <is>
           <t>nassira-propertie-12288954</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr">
+      <c r="B109" t="inlineStr">
         <is>
           <t>65102649106</t>
         </is>
       </c>
-      <c r="C108" s="2" t="inlineStr">
+      <c r="C109" s="2" t="inlineStr">
         <is>
           <t>https://www.propertyfinder.ae/en/plp/buy/villa-for-sale-dubai-dubai-hills-estate-sidra-villas-sidra-villas-iii-13283643.html</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr">
+      <c r="D109" t="inlineStr">
         <is>
           <t>Dubai Hills Estate</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
+      <c r="E109" t="inlineStr">
         <is>
           <t>Sidra Villas</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr">
+      <c r="F109" t="inlineStr">
         <is>
           <t>Sidra Villas III</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr">
+      <c r="G109" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H108" t="n">
+      <c r="H109" t="n">
         <v>9000000</v>
       </c>
-      <c r="I108" t="n">
+      <c r="I109" t="n">
         <v>3</v>
       </c>
-      <c r="J108" t="inlineStr">
+      <c r="J109" t="inlineStr">
         <is>
           <t>Villa</t>
         </is>
       </c>
-      <c r="K108" t="inlineStr">
+      <c r="K109" t="inlineStr">
         <is>
           <t>Type E1</t>
         </is>
       </c>
-      <c r="M108" t="inlineStr">
+      <c r="M109" t="inlineStr">
         <is>
           <t>3100</t>
         </is>
       </c>
-      <c r="N108" t="inlineStr">
+      <c r="N109" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="O108" t="inlineStr">
+      <c r="O109" t="inlineStr">
         <is>
           <t xml:space="preserve">Spacious l Plus Maid l A Perfect Family Community </t>
         </is>
       </c>
-      <c r="P108" t="inlineStr">
+      <c r="P109" t="inlineStr">
         <is>
           <t>2025-01-13</t>
         </is>
       </c>
-      <c r="Q108" t="n">
-        <v>205</v>
-      </c>
-      <c r="R108" t="inlineStr">
+      <c r="Q109" t="n">
+        <v>206</v>
+      </c>
+      <c r="R109" t="inlineStr">
         <is>
           <t>Nassira Sekkay</t>
         </is>
       </c>
-      <c r="S108" t="inlineStr">
+      <c r="S109" t="inlineStr">
         <is>
           <t>Nassira Realty Group</t>
         </is>
       </c>
-      <c r="T108" t="inlineStr">
+      <c r="T109" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
       </c>
-      <c r="U108" t="inlineStr">
+      <c r="U109" t="inlineStr">
         <is>
           <t xml:space="preserve">Nassira Properties is pleased to present this beautiful 3-bedroom villa in Sidra, Dubai Hills Estate.
 This spacious property features a naturally landscaped garden and a large plot, making it perfect for families. The villa is ideally located just a stone&amp;#39;s throw away from the pool, park, and entrance, offering convenient access to all amenities. The property is in immaculate condition, and viewings are highly recommended.
@@ -12275,92 +12385,92 @@
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" s="1" t="inlineStr">
+    <row r="110">
+      <c r="A110" s="1" t="inlineStr">
         <is>
           <t>sidra1-Dubai-Hills-Estate</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr">
+      <c r="B110" t="inlineStr">
         <is>
           <t>6528039898</t>
         </is>
       </c>
-      <c r="C109" s="2" t="inlineStr">
+      <c r="C110" s="2" t="inlineStr">
         <is>
           <t>https://www.propertyfinder.ae/en/plp/buy/villa-for-sale-dubai-dubai-hills-estate-sidra-villas-sidra-villas-i-14383967.html</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr">
+      <c r="D110" t="inlineStr">
         <is>
           <t>Dubai Hills Estate</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr">
+      <c r="E110" t="inlineStr">
         <is>
           <t>Sidra Villas</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr">
+      <c r="F110" t="inlineStr">
         <is>
           <t>Sidra Villas I</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr">
+      <c r="G110" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="H109" t="n">
+      <c r="H110" t="n">
         <v>25000000</v>
       </c>
-      <c r="I109" t="n">
+      <c r="I110" t="n">
         <v>7</v>
       </c>
-      <c r="J109" t="inlineStr">
+      <c r="J110" t="inlineStr">
         <is>
           <t>Villa</t>
         </is>
       </c>
-      <c r="M109" t="inlineStr">
+      <c r="M110" t="inlineStr">
         <is>
           <t>8117</t>
         </is>
       </c>
-      <c r="N109" t="inlineStr">
+      <c r="N110" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="O109" t="inlineStr">
+      <c r="O110" t="inlineStr">
         <is>
           <t xml:space="preserve">Exclusive 7 Bedrooms | Park View | Upgraded </t>
         </is>
       </c>
-      <c r="P109" t="inlineStr">
+      <c r="P110" t="inlineStr">
         <is>
           <t>2025-05-29</t>
         </is>
       </c>
-      <c r="Q109" t="n">
-        <v>69</v>
-      </c>
-      <c r="R109" t="inlineStr">
+      <c r="Q110" t="n">
+        <v>70</v>
+      </c>
+      <c r="R110" t="inlineStr">
         <is>
           <t>Wajahat Malik</t>
         </is>
       </c>
-      <c r="S109" t="inlineStr">
+      <c r="S110" t="inlineStr">
         <is>
           <t>BESTRONG REAL ESTATE BROKERAGE L.L.C</t>
         </is>
       </c>
-      <c r="T109" t="inlineStr">
+      <c r="T110" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
       </c>
-      <c r="U109" t="inlineStr">
+      <c r="U110" t="inlineStr">
         <is>
           <t xml:space="preserve">Experience true luxury living in this exceptionally upgraded 7-bedroom villa in the prestigious Sidra 1, Dubai Hills Estate. With a fully extended layout and elegant design, this home offers an ideal setting for comfort, privacy, and family living.
 Property Details:
@@ -12400,97 +12510,97 @@
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" s="1" t="inlineStr">
+    <row r="111">
+      <c r="A111" s="1" t="inlineStr">
         <is>
           <t>sisure-13062523-8c</t>
         </is>
       </c>
-      <c r="B110" s="3" t="inlineStr">
+      <c r="B111" s="3" t="inlineStr">
         <is>
           <t>65102648818</t>
         </is>
       </c>
-      <c r="C110" s="2" t="inlineStr">
+      <c r="C111" s="2" t="inlineStr">
         <is>
           <t>https://www.propertyfinder.ae/en/plp/buy/villa-for-sale-dubai-dubai-hills-estate-sidra-villas-sidra-villas-iii-14708222.html</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr">
+      <c r="D111" t="inlineStr">
         <is>
           <t>Dubai Hills Estate</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
+      <c r="E111" t="inlineStr">
         <is>
           <t>Sidra Villas</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr">
+      <c r="F111" t="inlineStr">
         <is>
           <t>Sidra Villas III</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr">
+      <c r="G111" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H110" t="n">
+      <c r="H111" t="n">
         <v>8500000</v>
       </c>
-      <c r="I110" t="n">
+      <c r="I111" t="n">
         <v>3</v>
       </c>
-      <c r="J110" t="inlineStr">
+      <c r="J111" t="inlineStr">
         <is>
           <t>Villa</t>
         </is>
       </c>
-      <c r="K110" t="inlineStr">
+      <c r="K111" t="inlineStr">
         <is>
           <t>Type E1</t>
         </is>
       </c>
-      <c r="M110" t="inlineStr">
+      <c r="M111" t="inlineStr">
         <is>
           <t>3100</t>
         </is>
       </c>
-      <c r="N110" t="inlineStr">
+      <c r="N111" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="O110" t="inlineStr">
+      <c r="O111" t="inlineStr">
         <is>
           <t>Corner | Serious Seller | Vastu</t>
         </is>
       </c>
-      <c r="P110" t="inlineStr">
+      <c r="P111" t="inlineStr">
         <is>
           <t>2025-07-09</t>
         </is>
       </c>
-      <c r="Q110" t="n">
-        <v>28</v>
-      </c>
-      <c r="R110" t="inlineStr">
+      <c r="Q111" t="n">
+        <v>29</v>
+      </c>
+      <c r="R111" t="inlineStr">
         <is>
           <t>Omar Zein</t>
         </is>
       </c>
-      <c r="S110" t="inlineStr">
+      <c r="S111" t="inlineStr">
         <is>
           <t>SISU REAL ESTATE L.L.C</t>
         </is>
       </c>
-      <c r="T110" t="inlineStr">
+      <c r="T111" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
       </c>
-      <c r="U110" t="inlineStr">
+      <c r="U111" t="inlineStr">
         <is>
           <t>Sisu Real Estate is delighted to present this modern 3 Bedrooms Villa at Sidra 3 - Dubai Hills Estate
 • Sidra 3 - Dubai Hills Estate
@@ -12520,97 +12630,97 @@
         </is>
       </c>
     </row>
-    <row r="111">
-      <c r="A111" s="1" t="inlineStr">
+    <row r="112">
+      <c r="A112" s="1" t="inlineStr">
         <is>
           <t>sycapital-14008540</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr">
+      <c r="B112" t="inlineStr">
         <is>
           <t>6544032282</t>
         </is>
       </c>
-      <c r="C111" s="2" t="inlineStr">
+      <c r="C112" s="2" t="inlineStr">
         <is>
           <t>https://www.propertyfinder.ae/en/plp/buy/villa-for-sale-dubai-dubai-hills-estate-sidra-villas-sidra-villas-ii-14539531.html</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr">
+      <c r="D112" t="inlineStr">
         <is>
           <t>Dubai Hills Estate</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr">
+      <c r="E112" t="inlineStr">
         <is>
           <t>Sidra Villas</t>
         </is>
       </c>
-      <c r="F111" t="inlineStr">
+      <c r="F112" t="inlineStr">
         <is>
           <t>Sidra Villas II</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr">
+      <c r="G112" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H111" t="n">
+      <c r="H112" t="n">
         <v>8500000</v>
       </c>
-      <c r="I111" t="n">
+      <c r="I112" t="n">
         <v>3</v>
       </c>
-      <c r="J111" t="inlineStr">
+      <c r="J112" t="inlineStr">
         <is>
           <t>Villa</t>
         </is>
       </c>
-      <c r="K111" t="inlineStr">
+      <c r="K112" t="inlineStr">
         <is>
           <t>Type E1</t>
         </is>
       </c>
-      <c r="M111" t="inlineStr">
+      <c r="M112" t="inlineStr">
         <is>
           <t>3100</t>
         </is>
       </c>
-      <c r="N111" t="inlineStr">
+      <c r="N112" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="O111" t="inlineStr">
+      <c r="O112" t="inlineStr">
         <is>
           <t>Spacious 3 Bedroom Villa | Landscaped Garden</t>
         </is>
       </c>
-      <c r="P111" t="inlineStr">
+      <c r="P112" t="inlineStr">
         <is>
           <t>2025-06-19</t>
         </is>
       </c>
-      <c r="Q111" t="n">
-        <v>48</v>
-      </c>
-      <c r="R111" t="inlineStr">
+      <c r="Q112" t="n">
+        <v>49</v>
+      </c>
+      <c r="R112" t="inlineStr">
         <is>
           <t>Muhammad Sajid</t>
         </is>
       </c>
-      <c r="S111" t="inlineStr">
+      <c r="S112" t="inlineStr">
         <is>
           <t>SY Capital Estates</t>
         </is>
       </c>
-      <c r="T111" t="inlineStr">
+      <c r="T112" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
       </c>
-      <c r="U111" t="inlineStr">
+      <c r="U112" t="inlineStr">
         <is>
           <t>Annuated interior to experience a tastefully interior that seamlessly combines modern design with everyday functionality.
 Sidra II is a master-planned community designed to cater to families seeking an exceptional lifestyle. This remarkable property is situated in a prime location within Sidra II, offering easy access to Dubai Hills Mall and The Golf Club, both just a short distance away.
@@ -12630,128 +12740,20 @@
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" s="4" t="inlineStr">
-        <is>
-          <t>L-9009</t>
-        </is>
-      </c>
-      <c r="B112" s="5" t="inlineStr">
-        <is>
-          <t>6529103221</t>
-        </is>
-      </c>
-      <c r="C112" s="2" t="inlineStr">
-        <is>
-          <t>https://www.propertyfinder.ae/en/plp/buy/villa-for-sale-dubai-dubai-hills-estate-sidra-villas-sidra-villas-i-14890412.html</t>
-        </is>
-      </c>
-      <c r="D112" s="5" t="inlineStr">
-        <is>
-          <t>Dubai Hills Estate</t>
-        </is>
-      </c>
-      <c r="E112" s="5" t="inlineStr">
-        <is>
-          <t>Sidra Villas</t>
-        </is>
-      </c>
-      <c r="F112" s="5" t="inlineStr">
-        <is>
-          <t>Sidra Villas I</t>
-        </is>
-      </c>
-      <c r="G112" s="5" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="H112" s="5" t="n">
-        <v>10500000</v>
-      </c>
-      <c r="I112" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="J112" s="5" t="inlineStr">
-        <is>
-          <t>Villa</t>
-        </is>
-      </c>
-      <c r="K112" s="5" t="inlineStr">
-        <is>
-          <t>Type E1</t>
-        </is>
-      </c>
-      <c r="L112" s="5" t="inlineStr"/>
-      <c r="M112" s="6" t="inlineStr">
-        <is>
-          <t>3100</t>
-        </is>
-      </c>
-      <c r="N112" s="5" t="inlineStr"/>
-      <c r="O112" s="5" t="inlineStr">
-        <is>
-          <t>Exclusive Luxury Villa | Private Pool | E1</t>
-        </is>
-      </c>
-      <c r="P112" s="5" t="inlineStr">
-        <is>
-          <t>2025-08-05</t>
-        </is>
-      </c>
-      <c r="Q112" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="R112" s="5" t="inlineStr">
-        <is>
-          <t>Peter Delargey</t>
-        </is>
-      </c>
-      <c r="S112" s="5" t="inlineStr">
-        <is>
-          <t>EQUITY REAL ESTATES L.L.C</t>
-        </is>
-      </c>
-      <c r="T112" s="5" t="inlineStr">
-        <is>
-          <t>Available</t>
-        </is>
-      </c>
-      <c r="U112" s="5" t="inlineStr">
-        <is>
-          <t>Equity wants you to experience a luxurious living space meticulously upgraded to offer an unparalleled lifestyle in Sidra Villa, Dubai Hills Estate.
-- 3 Bedroom + Maids
-- Fully Upgraded
-- Stunning Finishing
-- Highest Quality Upgrades
-- Single Road
-- Vacant On Transfer
-- Plot 4,486.61 Sq Ft
-- Open Plan Living, Kitchen and Dining
-- Permit No.: 6529103221
-The interior offers an extended living, kitchen, and dining area designed for both comfort and elegance, featuring a flush ceiling with modern lighting and pristine high-end furniture. A striking TV wall unit with a 3D fireplace adds warmth and sophistication, making it perfect for cozy gatherings.
-Step outside to a private outdoor sanctuary with a luxurious overflow pool, refreshing shower, and a stylish dining area complete with an electric awning for shade. A sleek aluminum pergola and marble-finished bar complete the space, ideal for relaxing or entertaining in style.
-Please be advised that all measurements and information are provided to the best of our knowledge. Equity disclaims any liability for inaccuracies or discrepancies.
-Equity
-RERA ORN: 43321
-Address: Office 1902, Boulevard Plaza Tower 2, Downtown Dubai, Dubai, UAE</t>
-        </is>
-      </c>
-    </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>luxure-14092927</t>
-        </is>
-      </c>
-      <c r="B113" s="5" t="inlineStr">
-        <is>
-          <t>65102648813</t>
+          <t>LP45886</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>6531921899</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>https://www.propertyfinder.ae/en/plp/buy/villa-for-sale-dubai-dubai-hills-estate-sidra-villas-sidra-villas-iii-14833599.html</t>
+          <t>https://www.propertyfinder.ae/en/plp/buy/villa-for-sale-dubai-dubai-hills-estate-sidra-villas-sidra-villas-i-14900575.html</t>
         </is>
       </c>
       <c r="D113" s="5" t="inlineStr">
@@ -12766,7 +12768,7 @@
       </c>
       <c r="F113" s="5" t="inlineStr">
         <is>
-          <t>Sidra Villas III</t>
+          <t>Sidra Villas I</t>
         </is>
       </c>
       <c r="G113" s="5" t="inlineStr">
@@ -12775,7 +12777,7 @@
         </is>
       </c>
       <c r="H113" s="5" t="n">
-        <v>15000000</v>
+        <v>13750000</v>
       </c>
       <c r="I113" s="5" t="n">
         <v>5</v>
@@ -12785,39 +12787,35 @@
           <t>Villa</t>
         </is>
       </c>
-      <c r="K113" s="5" t="inlineStr">
-        <is>
-          <t>Type E5</t>
-        </is>
-      </c>
+      <c r="K113" s="5" t="inlineStr"/>
       <c r="L113" s="5" t="inlineStr"/>
       <c r="M113" s="6" t="inlineStr">
         <is>
-          <t>4109</t>
+          <t>5652</t>
         </is>
       </c>
       <c r="N113" s="5" t="inlineStr"/>
       <c r="O113" s="5" t="inlineStr">
         <is>
-          <t>Fullly Upgraded | Furnished | Private Pool</t>
+          <t>Fully Upgraded | On Green Belt | High ROI</t>
         </is>
       </c>
       <c r="P113" s="5" t="inlineStr">
         <is>
-          <t>2025-07-28</t>
+          <t>2025-08-06</t>
         </is>
       </c>
       <c r="Q113" s="5" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="R113" s="5" t="inlineStr">
         <is>
-          <t>Hibildas Haridas</t>
+          <t>Andrew Newman</t>
         </is>
       </c>
       <c r="S113" s="5" t="inlineStr">
         <is>
-          <t>THE LUXURY REAL ESTATE BROKER L.L.C</t>
+          <t>LuxuryProperty.com</t>
         </is>
       </c>
       <c r="T113" s="5" t="inlineStr">
@@ -12827,20 +12825,119 @@
       </c>
       <c r="U113" s="5" t="inlineStr">
         <is>
-          <t>The Luxury Real Estate is thrilled to present this fully upgraded, spacious, and elegantly furnished 4-bedroom villa with a serene community view in Sidra III, developed by Emaar Properties.
-Property Features:
-- Five Bedrooms
-- Six Bathrooms
-- Size: 4,902.96 SqFt.
-- Balcony with Community View
-- 2 Covered Parking Spaces
-- Fully Upgraded
-- Fully Furnished
+          <t>&lt;p&gt;Luxuryproperty.com is proud to preset this 5 bedroom Villa with maid&amp;#39;s room. This villa is a prime example of Dubai luxurious family living based in the prestigious Sidra 1 community of Dubai Hills Estate. Spanning across 5,652.88 sqf.&lt;br&gt;&lt;br&gt; &lt;/p&gt;&lt;p&gt;Key Features:&lt;/p&gt;&lt;ul&gt;&lt;li&gt;5.82% ROI&lt;br&gt;Ideal location backing onto Sidra 2&lt;br&gt;Maids room plus 5 Bedrooms&lt;br&gt;Swimming pool &lt;br&gt;Sunken seating entertainment area next to pool&lt;br&gt;Fully enclosed garage (optional extra from build)&lt;br&gt;Large open plan living &amp;amp; dining space&lt;br&gt;Balcony overlooking the pool&lt;br&gt;Fully landscaped pool area and garden&lt;br&gt;Great investment opportunity. &lt;br&gt;Contract renews Q4, 2025&lt;/li&gt;&lt;/ul&gt;&lt;p&gt; &lt;/p&gt;&lt;p&gt;This unique investment opportunity can also be taken vacant possession if the buyer would want to live in the Villa rather than rent out.  This Villa in Sidra 1, located within Dubai Hills Estate, enjoys a prime position in this sought-after Emaar community.&lt;/p&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="4" t="inlineStr">
+        <is>
+          <t>VI9073</t>
+        </is>
+      </c>
+      <c r="B114" s="5" t="inlineStr">
+        <is>
+          <t>6544014240</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>https://www.propertyfinder.ae/en/plp/buy/villa-for-sale-dubai-dubai-hills-estate-sidra-villas-sidra-villas-ii-14901717.html</t>
+        </is>
+      </c>
+      <c r="D114" s="5" t="inlineStr">
+        <is>
+          <t>Dubai Hills Estate</t>
+        </is>
+      </c>
+      <c r="E114" s="5" t="inlineStr">
+        <is>
+          <t>Sidra Villas</t>
+        </is>
+      </c>
+      <c r="F114" s="5" t="inlineStr">
+        <is>
+          <t>Sidra Villas II</t>
+        </is>
+      </c>
+      <c r="G114" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H114" s="5" t="n">
+        <v>12000000</v>
+      </c>
+      <c r="I114" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="J114" s="5" t="inlineStr">
+        <is>
+          <t>Villa</t>
+        </is>
+      </c>
+      <c r="K114" s="5" t="inlineStr">
+        <is>
+          <t>Type E3</t>
+        </is>
+      </c>
+      <c r="L114" s="5" t="inlineStr"/>
+      <c r="M114" s="7" t="inlineStr">
+        <is>
+          <t>3533</t>
+        </is>
+      </c>
+      <c r="N114" s="5" t="inlineStr"/>
+      <c r="O114" s="5" t="inlineStr">
+        <is>
+          <t>Community Expert | Exclusive | Extended</t>
+        </is>
+      </c>
+      <c r="P114" s="5" t="inlineStr">
+        <is>
+          <t>2025-08-06</t>
+        </is>
+      </c>
+      <c r="Q114" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="R114" s="5" t="inlineStr">
+        <is>
+          <t>Ahlam Dourhi</t>
+        </is>
+      </c>
+      <c r="S114" s="5" t="inlineStr">
+        <is>
+          <t>Jade &amp; Co Real Estate</t>
+        </is>
+      </c>
+      <c r="T114" s="5" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+      <c r="U114" s="5" t="inlineStr">
+        <is>
+          <t>Jade &amp;amp; Co Real Estate is proud to present this stunning 4-bedroom villa in the highly desirable community of Sidra. This Type E3 home has been extended to its full potential, offering exceptional indoor and outdoor living spaces.
+- Exclusive 4 Bedrooms
+- Green Belt
+- Large Corner Plot
+- Maximum Extended
+- Enclosed Balconies
 - Private Pool
-- Bright &amp;amp; Spacious
-- Standard Layout
-Located in the prestigious Dubai Hills Estate, this villa offers a tranquil living experience, surrounded by nature&amp;#39;s beauty. The design of Sidra villas incorporates a minimalist architectural style, maximizing natural light and airflow, creating a harmonious and eco-friendly living environment. 
-The Luxury Real Estate (TLRE) is a premier global real estate company specializing in high-end properties. With access to an exclusively owned portfolio, TLRE offers unique, luxury residences to discerning buyers. known for its personalized service and extensive market expertise, it connects clients to exceptional homes worldwide.</t>
+- Fantastic Location
+- Private Gym
+- Electric Covered Garage
+- Pantry Kitchen 
+- Tenanted
+- For viewing schedules and queries please contact our Sidra Specialist Ahlam
+Set on the green belt, the villa enjoys privacy and serene surroundings. The garden is beautifully landscaped and features a private outdoor gym, inviting swimming pool, and charming seating area, ideal for entertaining.
+The entrance has been extended to create a grander, more welcoming hallway, while the courtyard has been enclosed and built up to G+1, completed prior to Emaar’s new extension regulations—a rare and valuable feature. Additionally, the maid’s room has been thoughtfully converted into a spacious pantry kitchen, enhancing functionality.
+Upstairs, the bedroom balconies have been extended, offering more usable space, and the master suite includes a generous walk-in wardrobe with a skylight, filling the space with natural light. This is a truly exceptional home that must be seen to be appreciated.
+Sidra is Dubai’s most vibrant and premium new community. Dubai Hills is strategically positioned on Al Khail Road and southeast of Downtown Dubai. 
+Jade &amp;amp; Co was founded to provide a boutique approach to the Dubai Real Estate market, which caters way beyond beautiful properties, as our exceptional agents source a lifestyle to compliment you. Our purpose is to provide an unrivaled service in the market, whether you are buying, selling, or renting, and our approach allows us to walk alongside our clients at every stage of their journey. 
+Jade &amp;amp; Co Real Estate
+Office: 610 The Onyx Tower 1, The Greens, Dubai, UAE</t>
         </is>
       </c>
     </row>
@@ -12959,6 +13056,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId110"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId111"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId113"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>